<commit_message>
fixed the pinout excel sheet and the according header declaration file
</commit_message>
<xml_diff>
--- a/schematics/Pinout.xlsx
+++ b/schematics/Pinout.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\coding\esp_led\schematics\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C61C8148-853F-4754-A0E4-6B17F352F6D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{611E5AD1-6E13-4D89-A924-3EA2D6FE1C72}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-345" yWindow="3840" windowWidth="28770" windowHeight="17250" xr2:uid="{7B709400-5527-4F09-B168-7ABD178E598D}"/>
+    <workbookView xWindow="-28920" yWindow="2220" windowWidth="29040" windowHeight="17520" xr2:uid="{7B709400-5527-4F09-B168-7ABD178E598D}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="42">
   <si>
     <t xml:space="preserve">VIN </t>
   </si>
@@ -159,16 +159,30 @@
   </si>
   <si>
     <t>Color Button</t>
+  </si>
+  <si>
+    <t>https://esp32.implrust.com/esp32-intro/pinout.html</t>
+  </si>
+  <si>
+    <t>Picture Source:</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -191,13 +205,16 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Link" xfId="1" builtinId="8"/>
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -217,23 +234,23 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>761999</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>66261</xdr:rowOff>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>19050</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>133350</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>116632</xdr:colOff>
-      <xdr:row>21</xdr:row>
-      <xdr:rowOff>47211</xdr:rowOff>
+      <xdr:colOff>407377</xdr:colOff>
+      <xdr:row>25</xdr:row>
+      <xdr:rowOff>47625</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="Grafik 2" descr="ESP32 DevKit v1 ESP-WROOM-32">
+        <xdr:cNvPr id="2" name="Grafik 1" descr="https://esp32.implrust.com/esp32-intro/pinout.html">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{DC4DEE8D-50C8-8E9C-570F-9DA42D43A631}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{FBDECD21-2A65-C31A-E210-97FB91E18159}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -256,8 +273,8 @@
       </xdr:blipFill>
       <xdr:spPr bwMode="auto">
         <a:xfrm>
-          <a:off x="5333999" y="256761"/>
-          <a:ext cx="7736633" cy="3790950"/>
+          <a:off x="5353050" y="133350"/>
+          <a:ext cx="8191500" cy="4676775"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -596,8 +613,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F45F5D78-4331-4D3B-A7EE-DA52A10E1EE0}">
-  <dimension ref="B3:F17"/>
+  <dimension ref="B3:I27"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="8" max="8" width="14.140625" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="3" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B3" t="s">
@@ -744,7 +764,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B17" t="s">
         <v>0</v>
       </c>
@@ -752,8 +772,19 @@
         <v>28</v>
       </c>
     </row>
+    <row r="27" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="H27" t="s">
+        <v>41</v>
+      </c>
+      <c r="I27" s="1" t="s">
+        <v>40</v>
+      </c>
+    </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="I27" r:id="rId1" xr:uid="{5BDFA4CD-54B6-4909-95FF-372073AF5520}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>